<commit_message>
feat: Implement meet management features including event imports, athlete registrations, and team management
- Added MeetImportMixin for importing events, athletes, and registrations with validation.
- Introduced MeetNoticeMixin for exporting personal result notices in XLSX and PDF formats.
- Created MeetResultMixin for handling result recording and automatic ranking.
- Developed MeetTeamMixin for team creation, member management, and querying teams.
- Implemented validators for input validation in meet services.
- Added MeetViewMixin for various data retrieval and export functionalities related to events, athletes, and results.
</commit_message>
<xml_diff>
--- a/app/static/notice_templates/personal_notice_template.xlsx
+++ b/app/static/notice_templates/personal_notice_template.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="13500"/>
+    <workbookView windowWidth="25600" windowHeight="12200"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$I$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$I$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1244,8 +1244,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4714875" y="1637030"/>
-          <a:ext cx="741680" cy="701675"/>
+          <a:off x="4801870" y="1610360"/>
+          <a:ext cx="755015" cy="681355"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1511,13 +1511,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:GX48"/>
-  <sheetFormatPr defaultColWidth="9.02777777777778" defaultRowHeight="14.4"/>
+  <dimension ref="A1:GX47"/>
+  <sheetFormatPr defaultColWidth="9.02727272727273" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="5.66666666666667" style="1" customWidth="1"/>
-    <col min="2" max="8" width="10.3888888888889" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.66666666666667" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.02777777777778" style="1"/>
+    <col min="1" max="1" width="5.66363636363636" style="1" customWidth="1"/>
+    <col min="2" max="8" width="10.3909090909091" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.66363636363636" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.02727272727273" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:206">
@@ -1728,7 +1728,7 @@
       <c r="GW1" s="3"/>
       <c r="GX1" s="3"/>
     </row>
-    <row r="2" ht="28.2" spans="1:206">
+    <row r="2" ht="27.5" spans="1:206">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1938,7 +1938,7 @@
       <c r="GW2" s="3"/>
       <c r="GX2" s="3"/>
     </row>
-    <row r="3" ht="20.4" spans="1:206">
+    <row r="3" ht="21" spans="1:206">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -4248,7 +4248,7 @@
       <c r="GW13" s="3"/>
       <c r="GX13" s="3"/>
     </row>
-    <row r="14" ht="17.4" spans="1:206">
+    <row r="14" ht="17.5" spans="1:206">
       <c r="A14" s="2"/>
       <c r="B14" s="9" t="s">
         <v>12</v>
@@ -4464,7 +4464,7 @@
       <c r="GW14" s="3"/>
       <c r="GX14" s="3"/>
     </row>
-    <row r="15" ht="17.4" spans="1:206">
+    <row r="15" ht="17.5" spans="1:206">
       <c r="A15" s="2"/>
       <c r="B15" s="15">
         <v>1</v>
@@ -4674,7 +4674,7 @@
       <c r="GW15" s="3"/>
       <c r="GX15" s="3"/>
     </row>
-    <row r="16" ht="17.4" spans="1:206">
+    <row r="16" ht="17.5" spans="1:206">
       <c r="A16" s="2"/>
       <c r="B16" s="15">
         <v>2</v>
@@ -4884,7 +4884,7 @@
       <c r="GW16" s="3"/>
       <c r="GX16" s="3"/>
     </row>
-    <row r="17" ht="17.4" spans="1:206">
+    <row r="17" ht="17.5" spans="1:206">
       <c r="A17" s="2"/>
       <c r="B17" s="15">
         <v>3</v>
@@ -5098,7 +5098,7 @@
       <c r="GW17" s="3"/>
       <c r="GX17" s="3"/>
     </row>
-    <row r="18" ht="17.4" spans="1:206">
+    <row r="18" ht="17.5" spans="1:206">
       <c r="A18" s="2"/>
       <c r="B18" s="15">
         <v>4</v>
@@ -5312,7 +5312,7 @@
       <c r="GW18" s="3"/>
       <c r="GX18" s="3"/>
     </row>
-    <row r="19" ht="17.4" spans="1:206">
+    <row r="19" ht="17.5" spans="1:206">
       <c r="A19" s="2"/>
       <c r="B19" s="15">
         <v>5</v>
@@ -5526,7 +5526,7 @@
       <c r="GW19" s="3"/>
       <c r="GX19" s="3"/>
     </row>
-    <row r="20" ht="17.4" spans="1:206">
+    <row r="20" ht="17.5" spans="1:206">
       <c r="A20" s="2"/>
       <c r="B20" s="15">
         <v>6</v>
@@ -5740,7 +5740,7 @@
       <c r="GW20" s="3"/>
       <c r="GX20" s="3"/>
     </row>
-    <row r="21" ht="17.4" spans="1:206">
+    <row r="21" ht="17.5" spans="1:206">
       <c r="A21" s="3"/>
       <c r="B21" s="15">
         <v>7</v>
@@ -5954,7 +5954,7 @@
       <c r="GW21" s="3"/>
       <c r="GX21" s="3"/>
     </row>
-    <row r="22" ht="17.4" spans="1:206">
+    <row r="22" ht="17.5" spans="1:206">
       <c r="A22" s="3"/>
       <c r="B22" s="21">
         <v>8</v>
@@ -11368,214 +11368,6 @@
       <c r="GW47" s="3"/>
       <c r="GX47" s="3"/>
     </row>
-    <row r="48" ht="28.2" spans="1:206">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="3"/>
-      <c r="K48" s="3"/>
-      <c r="L48" s="3"/>
-      <c r="M48" s="3"/>
-      <c r="N48" s="3"/>
-      <c r="O48" s="3"/>
-      <c r="P48" s="3"/>
-      <c r="Q48" s="3"/>
-      <c r="R48" s="3"/>
-      <c r="S48" s="3"/>
-      <c r="T48" s="3"/>
-      <c r="U48" s="3"/>
-      <c r="V48" s="3"/>
-      <c r="W48" s="3"/>
-      <c r="X48" s="3"/>
-      <c r="Y48" s="3"/>
-      <c r="Z48" s="3"/>
-      <c r="AA48" s="3"/>
-      <c r="AB48" s="3"/>
-      <c r="AC48" s="3"/>
-      <c r="AD48" s="3"/>
-      <c r="AE48" s="3"/>
-      <c r="AF48" s="3"/>
-      <c r="AG48" s="3"/>
-      <c r="AH48" s="3"/>
-      <c r="AI48" s="3"/>
-      <c r="AJ48" s="3"/>
-      <c r="AK48" s="3"/>
-      <c r="AL48" s="3"/>
-      <c r="AM48" s="3"/>
-      <c r="AN48" s="3"/>
-      <c r="AO48" s="3"/>
-      <c r="AP48" s="3"/>
-      <c r="AQ48" s="3"/>
-      <c r="AR48" s="3"/>
-      <c r="AS48" s="3"/>
-      <c r="AT48" s="3"/>
-      <c r="AU48" s="3"/>
-      <c r="AV48" s="3"/>
-      <c r="AW48" s="3"/>
-      <c r="AX48" s="3"/>
-      <c r="AY48" s="3"/>
-      <c r="AZ48" s="3"/>
-      <c r="BA48" s="3"/>
-      <c r="BB48" s="3"/>
-      <c r="BC48" s="3"/>
-      <c r="BD48" s="3"/>
-      <c r="BE48" s="3"/>
-      <c r="BF48" s="3"/>
-      <c r="BG48" s="3"/>
-      <c r="BH48" s="3"/>
-      <c r="BI48" s="3"/>
-      <c r="BJ48" s="3"/>
-      <c r="BK48" s="3"/>
-      <c r="BL48" s="3"/>
-      <c r="BM48" s="3"/>
-      <c r="BN48" s="3"/>
-      <c r="BO48" s="3"/>
-      <c r="BP48" s="3"/>
-      <c r="BQ48" s="3"/>
-      <c r="BR48" s="3"/>
-      <c r="BS48" s="3"/>
-      <c r="BT48" s="3"/>
-      <c r="BU48" s="3"/>
-      <c r="BV48" s="3"/>
-      <c r="BW48" s="3"/>
-      <c r="BX48" s="3"/>
-      <c r="BY48" s="3"/>
-      <c r="BZ48" s="3"/>
-      <c r="CA48" s="3"/>
-      <c r="CB48" s="3"/>
-      <c r="CC48" s="3"/>
-      <c r="CD48" s="3"/>
-      <c r="CE48" s="3"/>
-      <c r="CF48" s="3"/>
-      <c r="CG48" s="3"/>
-      <c r="CH48" s="3"/>
-      <c r="CI48" s="3"/>
-      <c r="CJ48" s="3"/>
-      <c r="CK48" s="3"/>
-      <c r="CL48" s="3"/>
-      <c r="CM48" s="3"/>
-      <c r="CN48" s="3"/>
-      <c r="CO48" s="3"/>
-      <c r="CP48" s="3"/>
-      <c r="CQ48" s="3"/>
-      <c r="CR48" s="3"/>
-      <c r="CS48" s="3"/>
-      <c r="CT48" s="3"/>
-      <c r="CU48" s="3"/>
-      <c r="CV48" s="3"/>
-      <c r="CW48" s="3"/>
-      <c r="CX48" s="3"/>
-      <c r="CY48" s="3"/>
-      <c r="CZ48" s="3"/>
-      <c r="DA48" s="3"/>
-      <c r="DB48" s="3"/>
-      <c r="DC48" s="3"/>
-      <c r="DD48" s="3"/>
-      <c r="DE48" s="3"/>
-      <c r="DF48" s="3"/>
-      <c r="DG48" s="3"/>
-      <c r="DH48" s="3"/>
-      <c r="DI48" s="3"/>
-      <c r="DJ48" s="3"/>
-      <c r="DK48" s="3"/>
-      <c r="DL48" s="3"/>
-      <c r="DM48" s="3"/>
-      <c r="DN48" s="3"/>
-      <c r="DO48" s="3"/>
-      <c r="DP48" s="3"/>
-      <c r="DQ48" s="3"/>
-      <c r="DR48" s="3"/>
-      <c r="DS48" s="3"/>
-      <c r="DT48" s="3"/>
-      <c r="DU48" s="3"/>
-      <c r="DV48" s="3"/>
-      <c r="DW48" s="3"/>
-      <c r="DX48" s="3"/>
-      <c r="DY48" s="3"/>
-      <c r="DZ48" s="3"/>
-      <c r="EA48" s="3"/>
-      <c r="EB48" s="3"/>
-      <c r="EC48" s="3"/>
-      <c r="ED48" s="3"/>
-      <c r="EE48" s="3"/>
-      <c r="EF48" s="3"/>
-      <c r="EG48" s="3"/>
-      <c r="EH48" s="3"/>
-      <c r="EI48" s="3"/>
-      <c r="EJ48" s="3"/>
-      <c r="EK48" s="3"/>
-      <c r="EL48" s="3"/>
-      <c r="EM48" s="3"/>
-      <c r="EN48" s="3"/>
-      <c r="EO48" s="3"/>
-      <c r="EP48" s="3"/>
-      <c r="EQ48" s="3"/>
-      <c r="ER48" s="3"/>
-      <c r="ES48" s="3"/>
-      <c r="ET48" s="3"/>
-      <c r="EU48" s="3"/>
-      <c r="EV48" s="3"/>
-      <c r="EW48" s="3"/>
-      <c r="EX48" s="3"/>
-      <c r="EY48" s="3"/>
-      <c r="EZ48" s="3"/>
-      <c r="FA48" s="3"/>
-      <c r="FB48" s="3"/>
-      <c r="FC48" s="3"/>
-      <c r="FD48" s="3"/>
-      <c r="FE48" s="3"/>
-      <c r="FF48" s="3"/>
-      <c r="FG48" s="3"/>
-      <c r="FH48" s="3"/>
-      <c r="FI48" s="3"/>
-      <c r="FJ48" s="3"/>
-      <c r="FK48" s="3"/>
-      <c r="FL48" s="3"/>
-      <c r="FM48" s="3"/>
-      <c r="FN48" s="3"/>
-      <c r="FO48" s="3"/>
-      <c r="FP48" s="3"/>
-      <c r="FQ48" s="3"/>
-      <c r="FR48" s="3"/>
-      <c r="FS48" s="3"/>
-      <c r="FT48" s="3"/>
-      <c r="FU48" s="3"/>
-      <c r="FV48" s="3"/>
-      <c r="FW48" s="3"/>
-      <c r="FX48" s="3"/>
-      <c r="FY48" s="3"/>
-      <c r="FZ48" s="3"/>
-      <c r="GA48" s="3"/>
-      <c r="GB48" s="3"/>
-      <c r="GC48" s="3"/>
-      <c r="GD48" s="3"/>
-      <c r="GE48" s="3"/>
-      <c r="GF48" s="3"/>
-      <c r="GG48" s="3"/>
-      <c r="GH48" s="3"/>
-      <c r="GI48" s="3"/>
-      <c r="GJ48" s="3"/>
-      <c r="GK48" s="3"/>
-      <c r="GL48" s="3"/>
-      <c r="GM48" s="3"/>
-      <c r="GN48" s="3"/>
-      <c r="GO48" s="3"/>
-      <c r="GP48" s="3"/>
-      <c r="GQ48" s="3"/>
-      <c r="GR48" s="3"/>
-      <c r="GS48" s="3"/>
-      <c r="GT48" s="3"/>
-      <c r="GU48" s="3"/>
-      <c r="GV48" s="3"/>
-      <c r="GW48" s="3"/>
-      <c r="GX48" s="3"/>
-    </row>
   </sheetData>
   <mergeCells count="20">
     <mergeCell ref="A2:I2"/>

</xml_diff>

<commit_message>
Add event progress template and update server scripts
- Created a new HTML template for event progress with filtering and checkbox functionality.
- Implemented JavaScript for loading, filtering, and saving event progress data.
- Added `run_dev.py` for local development server setup.
- Added `run_prod.py` for production server setup using Waitress.
</commit_message>
<xml_diff>
--- a/app/static/notice_templates/personal_notice_template.xlsx
+++ b/app/static/notice_templates/personal_notice_template.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
   <si>
     <t>北京信息科技大学校运会</t>
   </si>
@@ -41,10 +41,7 @@
     <t>教工男子甲组1500米决赛</t>
   </si>
   <si>
-    <t>地点/时间：</t>
-  </si>
-  <si>
-    <t>操场</t>
+    <t>制表: 体育信息与竞技社团</t>
   </si>
   <si>
     <t>日期：</t>
@@ -2573,13 +2570,11 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
@@ -2989,7 +2984,7 @@
     <row r="8" spans="1:206">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -3199,7 +3194,7 @@
     <row r="9" spans="1:206">
       <c r="A9" s="2"/>
       <c r="B9" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -3409,7 +3404,7 @@
     <row r="10" spans="1:206">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -3619,7 +3614,7 @@
     <row r="11" spans="1:206">
       <c r="A11" s="2"/>
       <c r="B11" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -3829,15 +3824,15 @@
     <row r="12" spans="1:206">
       <c r="A12" s="6"/>
       <c r="B12" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -4251,18 +4246,18 @@
     <row r="14" ht="17.5" spans="1:206">
       <c r="A14" s="2"/>
       <c r="B14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>14</v>
       </c>
       <c r="E14" s="11"/>
       <c r="F14" s="12"/>
       <c r="G14" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H14" s="14"/>
       <c r="I14" s="2"/>
@@ -4466,9 +4461,7 @@
     </row>
     <row r="15" ht="17.5" spans="1:206">
       <c r="A15" s="2"/>
-      <c r="B15" s="15">
-        <v>1</v>
-      </c>
+      <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
       <c r="E15" s="17"/>
@@ -4676,9 +4669,7 @@
     </row>
     <row r="16" ht="17.5" spans="1:206">
       <c r="A16" s="2"/>
-      <c r="B16" s="15">
-        <v>2</v>
-      </c>
+      <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="16"/>
       <c r="E16" s="17"/>
@@ -4886,14 +4877,12 @@
     </row>
     <row r="17" ht="17.5" spans="1:206">
       <c r="A17" s="2"/>
-      <c r="B17" s="15">
-        <v>3</v>
-      </c>
+      <c r="B17" s="15"/>
       <c r="C17" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
@@ -5100,14 +5089,12 @@
     </row>
     <row r="18" ht="17.5" spans="1:206">
       <c r="A18" s="2"/>
-      <c r="B18" s="15">
-        <v>4</v>
-      </c>
+      <c r="B18" s="15"/>
       <c r="C18" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E18" s="17"/>
       <c r="F18" s="18"/>
@@ -5314,14 +5301,12 @@
     </row>
     <row r="19" ht="17.5" spans="1:206">
       <c r="A19" s="2"/>
-      <c r="B19" s="15">
-        <v>5</v>
-      </c>
+      <c r="B19" s="15"/>
       <c r="C19" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E19" s="17"/>
       <c r="F19" s="18"/>
@@ -5528,14 +5513,12 @@
     </row>
     <row r="20" ht="17.5" spans="1:206">
       <c r="A20" s="2"/>
-      <c r="B20" s="15">
-        <v>6</v>
-      </c>
+      <c r="B20" s="15"/>
       <c r="C20" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E20" s="17"/>
       <c r="F20" s="18"/>
@@ -5742,14 +5725,12 @@
     </row>
     <row r="21" ht="17.5" spans="1:206">
       <c r="A21" s="3"/>
-      <c r="B21" s="15">
-        <v>7</v>
-      </c>
+      <c r="B21" s="15"/>
       <c r="C21" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E21" s="17"/>
       <c r="F21" s="18"/>
@@ -5956,14 +5937,12 @@
     </row>
     <row r="22" ht="17.5" spans="1:206">
       <c r="A22" s="3"/>
-      <c r="B22" s="21">
-        <v>8</v>
-      </c>
+      <c r="B22" s="21"/>
       <c r="C22" s="22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E22" s="23"/>
       <c r="F22" s="24"/>
@@ -11391,10 +11370,10 @@
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="G22:H22"/>
   </mergeCells>
-  <pageMargins left="0.751388888888889" right="0.751388888888889" top="0.780555555555556" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.751388888888889" right="0.751388888888889" top="0.779166666666667" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600"/>
   <headerFooter>
-    <oddFooter>&amp;L&amp;T&amp;C北京信息科技大学计统社团制作 &amp;R&amp;D</oddFooter>
+    <oddFooter>&amp;L&amp;T&amp;C北京信息科技大学体育信息与竞技社团制作 &amp;R&amp;D</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>